<commit_message>
Import Kettlebells (validées) + branchement du comparatif dédié
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQYooFqe2Ca9bkV6gqeZVS
</commit_message>
<xml_diff>
--- a/data/import/MuscuGuide_Base_Produits.xlsx
+++ b/data/import/MuscuGuide_Base_Produits.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7fe4e726a84d4ecc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="R7b5f62162fe34974"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="R9cec57baca004427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="R93688208b42f417f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="Rc34668e0f1974ff9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="R90f8366475ec45f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re3a09d93d4f94b04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="R4e3c4196cca148c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="Rae2c657b2ee64e14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="R7ff59f63b1bc4820"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="R00f7979a1bfe47ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="R76ad8f9768994f14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -435,7 +435,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4c1b41b7f9d243ce"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc938825c9b0f437b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -687,7 +687,7 @@
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:f>COUNTA(Produits!E4:E250)</x:f>
-        <x:v>33</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C4" s="12"/>
       <x:c r="D4" s="12" t="str">
@@ -747,7 +747,7 @@
       </x:c>
       <x:c r="B6" s="12" t="n">
         <x:f>COUNTIF(Produits!AG4:AG250,"Validé")</x:f>
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C6" s="12"/>
       <x:c r="D6" s="12" t="str">
@@ -807,7 +807,7 @@
       </x:c>
       <x:c r="B8" s="38" t="n">
         <x:f>IFERROR(AVERAGE(Produits!U4:U250),0)</x:f>
-        <x:v>89</x:v>
+        <x:v>89.25</x:v>
       </x:c>
       <x:c r="C8" s="12"/>
       <x:c r="D8" s="12" t="str">
@@ -1013,7 +1013,7 @@
       </x:c>
       <x:c r="E15" s="12" t="n">
         <x:f>COUNTIF(Produits!B:B,D15)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F15" s="12" t="n">
         <x:f>COUNTIFS(Produits!B:B,D15,Produits!H:H,"??????????")</x:f>
@@ -1021,7 +1021,7 @@
       </x:c>
       <x:c r="G15" s="12" t="n">
         <x:f>COUNTIFS(Produits!B:B,D15,Produits!AG:AG,"Validé")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H15" s="46" t="n">
         <x:f>IFERROR(F15/E15,0)</x:f>
@@ -1259,7 +1259,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1299c99b45ce4653"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60461de78beb45da"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -4466,133 +4466,309 @@
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="12"/>
-      <x:c r="B37" s="12"/>
-      <x:c r="C37" s="12"/>
-      <x:c r="D37" s="12"/>
-      <x:c r="E37" s="12"/>
-      <x:c r="F37" s="12"/>
-      <x:c r="G37" s="12"/>
-      <x:c r="H37" s="12"/>
-      <x:c r="I37" s="12"/>
+      <x:c r="A37" s="12" t="str">
+        <x:v>MG-KETT-001</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
+        <x:v>Kettlebells</x:v>
+      </x:c>
+      <x:c r="C37" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D37" s="12" t="str">
+        <x:v>Choix MuscuGuide</x:v>
+      </x:c>
+      <x:c r="E37" s="12" t="str">
+        <x:v>PROIRON Kettlebell 12 kg en néoprène</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
+        <x:v>PROIRON</x:v>
+      </x:c>
+      <x:c r="G37" s="12" t="str">
+        <x:v>12 kg — fonte monobloc — revêtement néoprène — poignée large</x:v>
+      </x:c>
+      <x:c r="H37" s="12" t="str">
+        <x:v>B09T9MY8L3</x:v>
+      </x:c>
+      <x:c r="I37" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B09T9MY8L3</x:v>
+      </x:c>
       <x:c r="J37" s="12"/>
       <x:c r="K37" s="12" t="str">
         <x:f>IF(OR(H37="",J37=""),"", "https://www.amazon.fr/dp/"&amp;H37&amp;"?tag="&amp;J37)</x:f>
       </x:c>
       <x:c r="L37" s="12"/>
       <x:c r="M37" s="36"/>
-      <x:c r="N37" s="12"/>
-      <x:c r="O37" s="12"/>
-      <x:c r="P37" s="12"/>
-      <x:c r="Q37" s="12"/>
-      <x:c r="R37" s="12"/>
-      <x:c r="S37" s="12"/>
-      <x:c r="T37" s="12"/>
-      <x:c r="U37" s="12" t="str">
+      <x:c r="N37" s="12" t="str">
+        <x:v>Performance</x:v>
+      </x:c>
+      <x:c r="O37" s="12" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P37" s="12" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="Q37" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R37" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="S37" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T37" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="U37" s="12" t="n">
         <x:f>IF(COUNTA(O37:T37)=0,"",SUM(O37:T37))</x:f>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="V37" s="12" t="str">
         <x:f>IF(U37="","",IF(U37&gt;=95,"Exceptionnel",IF(U37&gt;=90,"Excellent",IF(U37&gt;=85,"Très bon",IF(U37&gt;=80,"Bon",IF(U37&gt;=70,"Correct","À revoir"))))))</x:f>
-      </x:c>
-      <x:c r="W37" s="12"/>
-      <x:c r="X37" s="12"/>
-      <x:c r="Y37" s="12"/>
-      <x:c r="Z37" s="12"/>
-      <x:c r="AA37" s="12"/>
-      <x:c r="AB37" s="12"/>
-      <x:c r="AC37" s="12"/>
-      <x:c r="AD37" s="12"/>
-      <x:c r="AE37" s="38"/>
-      <x:c r="AF37" s="40"/>
-      <x:c r="AG37" s="12"/>
-      <x:c r="AH37" s="12"/>
-      <x:c r="AI37" s="12"/>
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="W37" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="X37" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Y37" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Z37" s="12" t="str">
+        <x:v>Une kettlebell polyvalente et bien finie pour progresser sur les swings, squats et exercices de renforcement à domicile.</x:v>
+      </x:c>
+      <x:c r="AA37" s="12" t="str">
+        <x:v>Fonte monobloc | Revêtement néoprène protecteur | Poignée large | Note Amazon élevée | Format 12 kg polyvalent</x:v>
+      </x:c>
+      <x:c r="AB37" s="12" t="str">
+        <x:v>Poids fixe | Moins adaptée aux grands débutants | Le néoprène peut s’user avec un usage très intensif</x:v>
+      </x:c>
+      <x:c r="AC37" s="12" t="str">
+        <x:v>Débutant à intermédiaire recherchant une kettlebell polyvalente pour le home gym</x:v>
+      </x:c>
+      <x:c r="AD37" s="12" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="AE37" s="38" t="n">
+        <x:v>4.8</x:v>
+      </x:c>
+      <x:c r="AF37" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="AG37" s="12" t="str">
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH37" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B09T9MY8L3</x:v>
+      </x:c>
+      <x:c r="AI37" s="12" t="str">
+        <x:v>ASIN, poids de 12 kg, matière néoprène, note Amazon 4,8/5 et 116 commentaires vérifiés le 05/08/2026.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="12"/>
-      <x:c r="B38" s="12"/>
-      <x:c r="C38" s="12"/>
-      <x:c r="D38" s="12"/>
-      <x:c r="E38" s="12"/>
-      <x:c r="F38" s="12"/>
-      <x:c r="G38" s="12"/>
-      <x:c r="H38" s="12"/>
-      <x:c r="I38" s="12"/>
+      <x:c r="A38" s="12" t="str">
+        <x:v>MG-KETT-002</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>Kettlebells</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D38" s="12" t="str">
+        <x:v>Meilleur rapport qualité/prix</x:v>
+      </x:c>
+      <x:c r="E38" s="12" t="str">
+        <x:v>Yes4All Kettlebell en fonte avec revêtement poudre</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
+        <x:v>Yes4All</x:v>
+      </x:c>
+      <x:c r="G38" s="12" t="str">
+        <x:v>Gamme 4 à 32 kg — fonte monobloc — poignée large</x:v>
+      </x:c>
+      <x:c r="H38" s="12" t="str">
+        <x:v>B0DNK2V1WR</x:v>
+      </x:c>
+      <x:c r="I38" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0DNK2V1WR</x:v>
+      </x:c>
       <x:c r="J38" s="12"/>
       <x:c r="K38" s="12" t="str">
         <x:f>IF(OR(H38="",J38=""),"", "https://www.amazon.fr/dp/"&amp;H38&amp;"?tag="&amp;J38)</x:f>
       </x:c>
       <x:c r="L38" s="12"/>
       <x:c r="M38" s="36"/>
-      <x:c r="N38" s="12"/>
-      <x:c r="O38" s="12"/>
-      <x:c r="P38" s="12"/>
-      <x:c r="Q38" s="12"/>
-      <x:c r="R38" s="12"/>
-      <x:c r="S38" s="12"/>
-      <x:c r="T38" s="12"/>
-      <x:c r="U38" s="12" t="str">
+      <x:c r="N38" s="12" t="str">
+        <x:v>Essentials</x:v>
+      </x:c>
+      <x:c r="O38" s="12" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P38" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q38" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R38" s="12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="S38" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="T38" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="U38" s="12" t="n">
         <x:f>IF(COUNTA(O38:T38)=0,"",SUM(O38:T38))</x:f>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="V38" s="12" t="str">
         <x:f>IF(U38="","",IF(U38&gt;=95,"Exceptionnel",IF(U38&gt;=90,"Excellent",IF(U38&gt;=85,"Très bon",IF(U38&gt;=80,"Bon",IF(U38&gt;=70,"Correct","À revoir"))))))</x:f>
-      </x:c>
-      <x:c r="W38" s="12"/>
-      <x:c r="X38" s="12"/>
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="W38" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="X38" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
       <x:c r="Y38" s="12"/>
-      <x:c r="Z38" s="12"/>
-      <x:c r="AA38" s="12"/>
-      <x:c r="AB38" s="12"/>
-      <x:c r="AC38" s="12"/>
-      <x:c r="AD38" s="12"/>
-      <x:c r="AE38" s="38"/>
-      <x:c r="AF38" s="40"/>
-      <x:c r="AG38" s="12"/>
-      <x:c r="AH38" s="12"/>
-      <x:c r="AI38" s="12"/>
+      <x:c r="Z38" s="12" t="str">
+        <x:v>Une gamme populaire et accessible, avec de nombreux poids disponibles et une finition poudre adaptée aux entraînements réguliers.</x:v>
+      </x:c>
+      <x:c r="AA38" s="12" t="str">
+        <x:v>Très bon rapport qualité/prix | Gamme 4 à 32 kg | 4,7/5 sur plus de 4 500 évaluations | Poignée large | Fonte sans soudure</x:v>
+      </x:c>
+      <x:c r="AB38" s="12" t="str">
+        <x:v>L’ASIN correspond à une variante légère | Finition moins premium | Disponibilité variable selon le poids</x:v>
+      </x:c>
+      <x:c r="AC38" s="12" t="str">
+        <x:v>Débutant à confirmé souhaitant choisir précisément son poids</x:v>
+      </x:c>
+      <x:c r="AD38" s="12" t="n">
+        <x:v>4566</x:v>
+      </x:c>
+      <x:c r="AE38" s="38" t="n">
+        <x:v>4.7</x:v>
+      </x:c>
+      <x:c r="AF38" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="AG38" s="12" t="str">
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH38" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0DNK2V1WR</x:v>
+      </x:c>
+      <x:c r="AI38" s="12" t="str">
+        <x:v>ASIN de la variante Amazon FR, note 4,7/5 et 4 566 évaluations vérifiés le 05/08/2026. La fiche produit regroupe une gamme de 4 à 32 kg.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="12"/>
-      <x:c r="B39" s="12"/>
-      <x:c r="C39" s="12"/>
-      <x:c r="D39" s="12"/>
-      <x:c r="E39" s="12"/>
-      <x:c r="F39" s="12"/>
-      <x:c r="G39" s="12"/>
-      <x:c r="H39" s="12"/>
-      <x:c r="I39" s="12"/>
+      <x:c r="A39" s="12" t="str">
+        <x:v>MG-KETT-003</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
+        <x:v>Kettlebells</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D39" s="12" t="str">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="E39" s="12" t="str">
+        <x:v>Kettlebell Kings Powder Coat 8 kg</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="str">
+        <x:v>Kettlebell Kings</x:v>
+      </x:c>
+      <x:c r="G39" s="12" t="str">
+        <x:v>8 kg — fonte moulée en une pièce — finition poudre — base usinée</x:v>
+      </x:c>
+      <x:c r="H39" s="12" t="str">
+        <x:v>B017WB2OHQ</x:v>
+      </x:c>
+      <x:c r="I39" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B017WB2OHQ</x:v>
+      </x:c>
       <x:c r="J39" s="12"/>
       <x:c r="K39" s="12" t="str">
         <x:f>IF(OR(H39="",J39=""),"", "https://www.amazon.fr/dp/"&amp;H39&amp;"?tag="&amp;J39)</x:f>
       </x:c>
       <x:c r="L39" s="12"/>
       <x:c r="M39" s="36"/>
-      <x:c r="N39" s="12"/>
-      <x:c r="O39" s="12"/>
-      <x:c r="P39" s="12"/>
-      <x:c r="Q39" s="12"/>
-      <x:c r="R39" s="12"/>
-      <x:c r="S39" s="12"/>
-      <x:c r="T39" s="12"/>
-      <x:c r="U39" s="12" t="str">
+      <x:c r="N39" s="12" t="str">
+        <x:v>Elite</x:v>
+      </x:c>
+      <x:c r="O39" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P39" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="Q39" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="R39" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="S39" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="T39" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="U39" s="12" t="n">
         <x:f>IF(COUNTA(O39:T39)=0,"",SUM(O39:T39))</x:f>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="V39" s="12" t="str">
         <x:f>IF(U39="","",IF(U39&gt;=95,"Exceptionnel",IF(U39&gt;=90,"Excellent",IF(U39&gt;=85,"Très bon",IF(U39&gt;=80,"Bon",IF(U39&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="W39" s="12"/>
-      <x:c r="X39" s="12"/>
-      <x:c r="Y39" s="12"/>
-      <x:c r="Z39" s="12"/>
-      <x:c r="AA39" s="12"/>
-      <x:c r="AB39" s="12"/>
-      <x:c r="AC39" s="12"/>
-      <x:c r="AD39" s="12"/>
-      <x:c r="AE39" s="38"/>
-      <x:c r="AF39" s="40"/>
-      <x:c r="AG39" s="12"/>
-      <x:c r="AH39" s="12"/>
-      <x:c r="AI39" s="12"/>
+      <x:c r="X39" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Y39" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Z39" s="12" t="str">
+        <x:v>Une kettlebell premium en fonte monobloc, conçue pour une prise fiable et une grande durabilité lors des entraînements techniques.</x:v>
+      </x:c>
+      <x:c r="AA39" s="12" t="str">
+        <x:v>Fonte moulée en une pièce | Finition poudre durable | Base plane usinée | Très bonne prise en main | Fabrication précise</x:v>
+      </x:c>
+      <x:c r="AB39" s="12" t="str">
+        <x:v>Prix plus élevé | Poids fixe de 8 kg sur cet ASIN | Disponibilité parfois limitée</x:v>
+      </x:c>
+      <x:c r="AC39" s="12" t="str">
+        <x:v>Intermédiaire à confirmé privilégiant la qualité de fabrication et la durabilité</x:v>
+      </x:c>
+      <x:c r="AD39" s="12" t="n">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="AE39" s="38" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="AF39" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="AG39" s="12" t="str">
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH39" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B017WB2OHQ</x:v>
+      </x:c>
+      <x:c r="AI39" s="12" t="str">
+        <x:v>ASIN, modèle 8 kg, note Amazon 4,5/5 et 354 évaluations vérifiés le 05/08/2026. Fonte monobloc, finition poudre et base plane confirmées sur la fiche Amazon FR.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="12"/>
@@ -13737,7 +13913,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c9c29d655b84855"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c2e6940412c4221"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16457,37 +16633,37 @@
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="12" t="n">
+      <x:c r="A37" s="12" t="str">
         <x:f>Produits!A37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B37" s="12" t="n">
+        <x:v>MG-KETT-001</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
         <x:f>Produits!B37</x:f>
-        <x:v>0</x:v>
+        <x:v>Kettlebells</x:v>
       </x:c>
       <x:c r="C37" s="12" t="n">
         <x:f>Produits!C37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D37" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D37" s="12" t="str">
         <x:f>Produits!D37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E37" s="12" t="n">
+        <x:v>Choix MuscuGuide</x:v>
+      </x:c>
+      <x:c r="E37" s="12" t="str">
         <x:f>Produits!E37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F37" s="12" t="n">
+        <x:v>PROIRON Kettlebell 12 kg en néoprène</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
         <x:f>Produits!F37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G37" s="12" t="n">
+        <x:v>PROIRON</x:v>
+      </x:c>
+      <x:c r="G37" s="12" t="str">
         <x:f>Produits!H37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H37" s="12" t="n">
+        <x:v>B09T9MY8L3</x:v>
+      </x:c>
+      <x:c r="H37" s="12" t="str">
         <x:f>Produits!I37</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B09T9MY8L3</x:v>
       </x:c>
       <x:c r="I37" s="12" t="n">
         <x:f>Produits!K37</x:f>
@@ -16499,65 +16675,65 @@
       </x:c>
       <x:c r="K37" s="12" t="n">
         <x:f>Produits!U37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L37" s="12" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="L37" s="12" t="str">
         <x:f>Produits!V37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M37" s="12" t="n">
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="M37" s="12" t="str">
         <x:f>Produits!Z37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N37" s="12" t="n">
+        <x:v>Une kettlebell polyvalente et bien finie pour progresser sur les swings, squats et exercices de renforcement à domicile.</x:v>
+      </x:c>
+      <x:c r="N37" s="12" t="str">
         <x:f>Produits!AA37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O37" s="12" t="n">
+        <x:v>Fonte monobloc | Revêtement néoprène protecteur | Poignée large | Note Amazon élevée | Format 12 kg polyvalent</x:v>
+      </x:c>
+      <x:c r="O37" s="12" t="str">
         <x:f>Produits!AB37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P37" s="12" t="n">
+        <x:v>Poids fixe | Moins adaptée aux grands débutants | Le néoprène peut s’user avec un usage très intensif</x:v>
+      </x:c>
+      <x:c r="P37" s="12" t="str">
         <x:f>Produits!AC37</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q37" s="12" t="n">
+        <x:v>Débutant à intermédiaire recherchant une kettlebell polyvalente pour le home gym</x:v>
+      </x:c>
+      <x:c r="Q37" s="12" t="str">
         <x:f>Produits!AG37</x:f>
-        <x:v>0</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="12" t="n">
+      <x:c r="A38" s="12" t="str">
         <x:f>Produits!A38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B38" s="12" t="n">
+        <x:v>MG-KETT-002</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
         <x:f>Produits!B38</x:f>
-        <x:v>0</x:v>
+        <x:v>Kettlebells</x:v>
       </x:c>
       <x:c r="C38" s="12" t="n">
         <x:f>Produits!C38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D38" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D38" s="12" t="str">
         <x:f>Produits!D38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E38" s="12" t="n">
+        <x:v>Meilleur rapport qualité/prix</x:v>
+      </x:c>
+      <x:c r="E38" s="12" t="str">
         <x:f>Produits!E38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F38" s="12" t="n">
+        <x:v>Yes4All Kettlebell en fonte avec revêtement poudre</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
         <x:f>Produits!F38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G38" s="12" t="n">
+        <x:v>Yes4All</x:v>
+      </x:c>
+      <x:c r="G38" s="12" t="str">
         <x:f>Produits!H38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H38" s="12" t="n">
+        <x:v>B0DNK2V1WR</x:v>
+      </x:c>
+      <x:c r="H38" s="12" t="str">
         <x:f>Produits!I38</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B0DNK2V1WR</x:v>
       </x:c>
       <x:c r="I38" s="12" t="n">
         <x:f>Produits!K38</x:f>
@@ -16569,65 +16745,65 @@
       </x:c>
       <x:c r="K38" s="12" t="n">
         <x:f>Produits!U38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L38" s="12" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="L38" s="12" t="str">
         <x:f>Produits!V38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M38" s="12" t="n">
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="M38" s="12" t="str">
         <x:f>Produits!Z38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N38" s="12" t="n">
+        <x:v>Une gamme populaire et accessible, avec de nombreux poids disponibles et une finition poudre adaptée aux entraînements réguliers.</x:v>
+      </x:c>
+      <x:c r="N38" s="12" t="str">
         <x:f>Produits!AA38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O38" s="12" t="n">
+        <x:v>Très bon rapport qualité/prix | Gamme 4 à 32 kg | 4,7/5 sur plus de 4 500 évaluations | Poignée large | Fonte sans soudure</x:v>
+      </x:c>
+      <x:c r="O38" s="12" t="str">
         <x:f>Produits!AB38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P38" s="12" t="n">
+        <x:v>L’ASIN correspond à une variante légère | Finition moins premium | Disponibilité variable selon le poids</x:v>
+      </x:c>
+      <x:c r="P38" s="12" t="str">
         <x:f>Produits!AC38</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q38" s="12" t="n">
+        <x:v>Débutant à confirmé souhaitant choisir précisément son poids</x:v>
+      </x:c>
+      <x:c r="Q38" s="12" t="str">
         <x:f>Produits!AG38</x:f>
-        <x:v>0</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="12" t="n">
+      <x:c r="A39" s="12" t="str">
         <x:f>Produits!A39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B39" s="12" t="n">
+        <x:v>MG-KETT-003</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
         <x:f>Produits!B39</x:f>
-        <x:v>0</x:v>
+        <x:v>Kettlebells</x:v>
       </x:c>
       <x:c r="C39" s="12" t="n">
         <x:f>Produits!C39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D39" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D39" s="12" t="str">
         <x:f>Produits!D39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E39" s="12" t="n">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="E39" s="12" t="str">
         <x:f>Produits!E39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F39" s="12" t="n">
+        <x:v>Kettlebell Kings Powder Coat 8 kg</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="str">
         <x:f>Produits!F39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G39" s="12" t="n">
+        <x:v>Kettlebell Kings</x:v>
+      </x:c>
+      <x:c r="G39" s="12" t="str">
         <x:f>Produits!H39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H39" s="12" t="n">
+        <x:v>B017WB2OHQ</x:v>
+      </x:c>
+      <x:c r="H39" s="12" t="str">
         <x:f>Produits!I39</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B017WB2OHQ</x:v>
       </x:c>
       <x:c r="I39" s="12" t="n">
         <x:f>Produits!K39</x:f>
@@ -16639,31 +16815,31 @@
       </x:c>
       <x:c r="K39" s="12" t="n">
         <x:f>Produits!U39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L39" s="12" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="L39" s="12" t="str">
         <x:f>Produits!V39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M39" s="12" t="n">
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="M39" s="12" t="str">
         <x:f>Produits!Z39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N39" s="12" t="n">
+        <x:v>Une kettlebell premium en fonte monobloc, conçue pour une prise fiable et une grande durabilité lors des entraînements techniques.</x:v>
+      </x:c>
+      <x:c r="N39" s="12" t="str">
         <x:f>Produits!AA39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O39" s="12" t="n">
+        <x:v>Fonte moulée en une pièce | Finition poudre durable | Base plane usinée | Très bonne prise en main | Fabrication précise</x:v>
+      </x:c>
+      <x:c r="O39" s="12" t="str">
         <x:f>Produits!AB39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P39" s="12" t="n">
+        <x:v>Prix plus élevé | Poids fixe de 8 kg sur cet ASIN | Disponibilité parfois limitée</x:v>
+      </x:c>
+      <x:c r="P39" s="12" t="str">
         <x:f>Produits!AC39</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q39" s="12" t="n">
+        <x:v>Intermédiaire à confirmé privilégiant la qualité de fabrication et la durabilité</x:v>
+      </x:c>
+      <x:c r="Q39" s="12" t="str">
         <x:f>Produits!AG39</x:f>
-        <x:v>0</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="40">

</xml_diff>

<commit_message>
Import Barres de traction (validées) + branchement du comparatif dédié
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQYooFqe2Ca9bkV6gqeZVS
</commit_message>
<xml_diff>
--- a/data/import/MuscuGuide_Base_Produits.xlsx
+++ b/data/import/MuscuGuide_Base_Produits.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re3a09d93d4f94b04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="R4e3c4196cca148c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="Rae2c657b2ee64e14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="R7ff59f63b1bc4820"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="R00f7979a1bfe47ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="R76ad8f9768994f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R539c652a54024d3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="R64f6e295511b429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="Rdc3186bfebd043f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="Rdc2e9e86ec46411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="Ra4b4f8a93f0d4617"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="Rb1b39ccfcf3c44d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -435,7 +435,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc938825c9b0f437b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R49611829e2f44a32"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -747,7 +747,7 @@
       </x:c>
       <x:c r="B6" s="12" t="n">
         <x:f>COUNTIF(Produits!AG4:AG250,"Validé")</x:f>
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C6" s="12"/>
       <x:c r="D6" s="12" t="str">
@@ -777,7 +777,7 @@
       </x:c>
       <x:c r="B7" s="12" t="n">
         <x:f>COUNTIF(Produits!AG4:AG250,"À rechercher")</x:f>
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="12"/>
       <x:c r="D7" s="12" t="str">
@@ -807,7 +807,7 @@
       </x:c>
       <x:c r="B8" s="38" t="n">
         <x:f>IFERROR(AVERAGE(Produits!U4:U250),0)</x:f>
-        <x:v>89.25</x:v>
+        <x:v>89.33333333333333</x:v>
       </x:c>
       <x:c r="C8" s="12"/>
       <x:c r="D8" s="12" t="str">
@@ -1208,7 +1208,7 @@
       </x:c>
       <x:c r="G22" s="12" t="n">
         <x:f>COUNTIFS(Produits!B:B,D22,Produits!AG:AG,"Validé")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H22" s="46" t="n">
         <x:f>IFERROR(F22/E22,0)</x:f>
@@ -1259,7 +1259,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60461de78beb45da"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a2e06aea0545b2"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -3345,14 +3345,20 @@
         <x:v>Choix MuscuGuide</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>KS300</x:v>
+        <x:v>Sportstech KS350</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
         <x:v>Sportstech</x:v>
       </x:c>
-      <x:c r="G25" s="12" t="str"/>
-      <x:c r="H25" s="12" t="str"/>
-      <x:c r="I25" s="12" t="str"/>
+      <x:c r="G25" s="12" t="str">
+        <x:v>Barre murale pliable — 3 prises — 3 œillets — charge utilisateur jusqu’à 150 kg</x:v>
+      </x:c>
+      <x:c r="H25" s="12" t="str">
+        <x:v>B0843FTZ9T</x:v>
+      </x:c>
+      <x:c r="I25" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0843FTZ9T</x:v>
+      </x:c>
       <x:c r="J25" s="12" t="str"/>
       <x:c r="K25" s="12" t="str">
         <x:f>IF(OR(H25="",J25=""),"", "https://www.amazon.fr/dp/"&amp;H25&amp;"?tag="&amp;J25)</x:f>
@@ -3362,17 +3368,31 @@
       <x:c r="N25" s="12" t="str">
         <x:v>Performance</x:v>
       </x:c>
-      <x:c r="O25" s="12" t="str"/>
-      <x:c r="P25" s="12" t="str"/>
-      <x:c r="Q25" s="12" t="str"/>
-      <x:c r="R25" s="12" t="str"/>
-      <x:c r="S25" s="12" t="str"/>
-      <x:c r="T25" s="12" t="str"/>
-      <x:c r="U25" s="12" t="str">
+      <x:c r="O25" s="12" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P25" s="12" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="Q25" s="12" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="R25" s="12" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="S25" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T25" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="U25" s="12" t="n">
         <x:f>IF(COUNTA(O25:T25)=0,"",SUM(O25:T25))</x:f>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="V25" s="12" t="str">
         <x:f>IF(U25="","",IF(U25&gt;=95,"Exceptionnel",IF(U25&gt;=90,"Excellent",IF(U25&gt;=85,"Très bon",IF(U25&gt;=80,"Bon",IF(U25&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="W25" s="12" t="str">
         <x:v>Oui</x:v>
@@ -3384,26 +3404,30 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="Z25" s="12" t="str">
-        <x:v>Barre polyvalente pour entraînement du haut du corps.</x:v>
+        <x:v>Une barre murale pliable, stable et polyvalente, particulièrement adaptée à un home gym compact.</x:v>
       </x:c>
       <x:c r="AA25" s="12" t="str">
-        <x:v>Multiprises | Polyvalence | Marque connue</x:v>
+        <x:v>Structure acier triangulaire | Pliable jusqu’à 26 cm | 3 positions de prise | 3 œillets d’entraînement | Kit de fixation inclus</x:v>
       </x:c>
       <x:c r="AB25" s="12" t="str">
-        <x:v>Compatibilité porte à vérifier</x:v>
+        <x:v>Perçage obligatoire | Mur solide indispensable | Moins mobile qu’un modèle de porte</x:v>
       </x:c>
       <x:c r="AC25" s="12" t="str">
-        <x:v>Home gym</x:v>
-      </x:c>
-      <x:c r="AD25" s="12" t="str"/>
-      <x:c r="AE25" s="38" t="str"/>
-      <x:c r="AF25" s="40" t="str"/>
+        <x:v>Débutant à confirmé recherchant une barre murale complète et peu encombrante</x:v>
+      </x:c>
+      <x:c r="AD25" s="12"/>
+      <x:c r="AE25" s="38"/>
+      <x:c r="AF25" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
       <x:c r="AG25" s="12" t="str">
-        <x:v>À rechercher</x:v>
-      </x:c>
-      <x:c r="AH25" s="12" t="str"/>
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH25" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0843FTZ9T</x:v>
+      </x:c>
       <x:c r="AI25" s="12" t="str">
-        <x:v>Vérifier version exacte.</x:v>
+        <x:v>ASIN Amazon FR vérifié le 05/08/2026. Sportstech confirme une structure acier, 3 prises, 3 œillets, un pliage à 26 cm et une charge utilisateur jusqu’à 150 kg. Note Amazon laissée vide faute de valeur FR suffisamment fiable.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -3420,14 +3444,20 @@
         <x:v>Meilleur rapport qualité/prix</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>Wall Mounted Pull-Up Bar</x:v>
+        <x:v>ONETWOFIT OT103</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
         <x:v>ONETWOFIT</x:v>
       </x:c>
-      <x:c r="G26" s="12" t="str"/>
-      <x:c r="H26" s="12" t="str"/>
-      <x:c r="I26" s="12" t="str"/>
+      <x:c r="G26" s="12" t="str">
+        <x:v>Barre de traction murale — conception 6 trous — charge annoncée jusqu’à 200 kg</x:v>
+      </x:c>
+      <x:c r="H26" s="12" t="str">
+        <x:v>B08K3Q74DR</x:v>
+      </x:c>
+      <x:c r="I26" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B08K3Q74DR</x:v>
+      </x:c>
       <x:c r="J26" s="12" t="str"/>
       <x:c r="K26" s="12" t="str">
         <x:f>IF(OR(H26="",J26=""),"", "https://www.amazon.fr/dp/"&amp;H26&amp;"?tag="&amp;J26)</x:f>
@@ -3437,17 +3467,31 @@
       <x:c r="N26" s="12" t="str">
         <x:v>Essentials</x:v>
       </x:c>
-      <x:c r="O26" s="12" t="str"/>
-      <x:c r="P26" s="12" t="str"/>
-      <x:c r="Q26" s="12" t="str"/>
-      <x:c r="R26" s="12" t="str"/>
-      <x:c r="S26" s="12" t="str"/>
-      <x:c r="T26" s="12" t="str"/>
-      <x:c r="U26" s="12" t="str">
+      <x:c r="O26" s="12" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="P26" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q26" s="12" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="R26" s="12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="S26" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="T26" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="U26" s="12" t="n">
         <x:f>IF(COUNTA(O26:T26)=0,"",SUM(O26:T26))</x:f>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="V26" s="12" t="str">
         <x:f>IF(U26="","",IF(U26&gt;=95,"Exceptionnel",IF(U26&gt;=90,"Excellent",IF(U26&gt;=85,"Très bon",IF(U26&gt;=80,"Bon",IF(U26&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Très bon</x:v>
       </x:c>
       <x:c r="W26" s="12" t="str">
         <x:v>Oui</x:v>
@@ -3459,26 +3503,32 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="Z26" s="12" t="str">
-        <x:v>Barre murale robuste à prix compétitif.</x:v>
+        <x:v>Une barre murale robuste et accessible, conçue pour offrir une fixation stable sans payer le prix d’un modèle premium.</x:v>
       </x:c>
       <x:c r="AA26" s="12" t="str">
-        <x:v>Stabilité | Multiprises | Prix</x:v>
+        <x:v>Excellent rapport qualité/prix | Conception 6 trous | Multiprises | Utilisation intérieure ou extérieure | Structure acier</x:v>
       </x:c>
       <x:c r="AB26" s="12" t="str">
-        <x:v>Installation avec perçage</x:v>
+        <x:v>Montage mural obligatoire | Qualité des chevilles à adapter au support | Finitions plus simples</x:v>
       </x:c>
       <x:c r="AC26" s="12" t="str">
-        <x:v>Débutant à confirmé</x:v>
-      </x:c>
-      <x:c r="AD26" s="12" t="str"/>
-      <x:c r="AE26" s="38" t="str"/>
-      <x:c r="AF26" s="40" t="str"/>
+        <x:v>Débutant à intermédiaire souhaitant une solution murale économique</x:v>
+      </x:c>
+      <x:c r="AD26" s="12"/>
+      <x:c r="AE26" s="38" t="n">
+        <x:v>4.3</x:v>
+      </x:c>
+      <x:c r="AF26" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
       <x:c r="AG26" s="12" t="str">
-        <x:v>À rechercher</x:v>
-      </x:c>
-      <x:c r="AH26" s="12" t="str"/>
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH26" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B08K3Q74DR</x:v>
+      </x:c>
       <x:c r="AI26" s="12" t="str">
-        <x:v>Vérifier charge max et fixations.</x:v>
+        <x:v>ASIN Amazon FR et note 4,3/5 vérifiés le 05/08/2026. Conception murale à 6 trous et charge annoncée jusqu’à 200 kg confirmées dans les résultats Amazon. Nombre d’évaluations laissé vide.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -3495,14 +3545,20 @@
         <x:v>Premium</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>Pull-Up &amp; Dip Bar</x:v>
+        <x:v>PULLUP &amp; DIP Barre de traction porte + station de dips</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>Pullup &amp; Dip</x:v>
-      </x:c>
-      <x:c r="G27" s="12" t="str"/>
-      <x:c r="H27" s="12" t="str"/>
-      <x:c r="I27" s="12" t="str"/>
+        <x:v>PULLUP &amp; DIP</x:v>
+      </x:c>
+      <x:c r="G27" s="12" t="str">
+        <x:v>Sans perçage — 4 prises — cadre 70 à 95 cm — charge jusqu’à 110 kg</x:v>
+      </x:c>
+      <x:c r="H27" s="12" t="str">
+        <x:v>B0CGDTN9VC</x:v>
+      </x:c>
+      <x:c r="I27" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0CGDTN9VC</x:v>
+      </x:c>
       <x:c r="J27" s="12" t="str"/>
       <x:c r="K27" s="12" t="str">
         <x:f>IF(OR(H27="",J27=""),"", "https://www.amazon.fr/dp/"&amp;H27&amp;"?tag="&amp;J27)</x:f>
@@ -3512,17 +3568,31 @@
       <x:c r="N27" s="12" t="str">
         <x:v>Elite</x:v>
       </x:c>
-      <x:c r="O27" s="12" t="str"/>
-      <x:c r="P27" s="12" t="str"/>
-      <x:c r="Q27" s="12" t="str"/>
-      <x:c r="R27" s="12" t="str"/>
-      <x:c r="S27" s="12" t="str"/>
-      <x:c r="T27" s="12" t="str"/>
-      <x:c r="U27" s="12" t="str">
+      <x:c r="O27" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="P27" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="Q27" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="R27" s="12" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="S27" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T27" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U27" s="12" t="n">
         <x:f>IF(COUNTA(O27:T27)=0,"",SUM(O27:T27))</x:f>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="V27" s="12" t="str">
         <x:f>IF(U27="","",IF(U27&gt;=95,"Exceptionnel",IF(U27&gt;=90,"Excellent",IF(U27&gt;=85,"Très bon",IF(U27&gt;=80,"Bon",IF(U27&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="W27" s="12" t="str"/>
       <x:c r="X27" s="12" t="str">
@@ -3532,26 +3602,34 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="Z27" s="12" t="str">
-        <x:v>Solution premium pour calisthénie et usage intensif.</x:v>
+        <x:v>Une solution premium sans perçage qui combine tractions et dips, idéale pour la calisthénie à domicile.</x:v>
       </x:c>
       <x:c r="AA27" s="12" t="str">
-        <x:v>Finition | Polyvalence | Stabilité</x:v>
+        <x:v>Aucun perçage | Barre de dips incluse | 4 positions de prise | Garantie 5 ans | Montage et retrait rapides</x:v>
       </x:c>
       <x:c r="AB27" s="12" t="str">
-        <x:v>Prix élevé</x:v>
+        <x:v>Prix élevé | Compatibilité du cadre de porte à vérifier | Charge limitée à 110 kg</x:v>
       </x:c>
       <x:c r="AC27" s="12" t="str">
-        <x:v>Calisthénie / confirmé</x:v>
-      </x:c>
-      <x:c r="AD27" s="12" t="str"/>
-      <x:c r="AE27" s="38" t="str"/>
-      <x:c r="AF27" s="40" t="str"/>
+        <x:v>Intermédiaire à confirmé pratiquant la calisthénie ou vivant en location</x:v>
+      </x:c>
+      <x:c r="AD27" s="12" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="AE27" s="38" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="AF27" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
       <x:c r="AG27" s="12" t="str">
-        <x:v>À rechercher</x:v>
-      </x:c>
-      <x:c r="AH27" s="12" t="str"/>
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH27" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0CGDTN9VC</x:v>
+      </x:c>
       <x:c r="AI27" s="12" t="str">
-        <x:v>Identifier modèle mural ou extérieur exact.</x:v>
+        <x:v>ASIN, note Amazon 4,5/5 et 400 évaluations vérifiés le 05/08/2026. Pullup &amp; Dip confirme l’installation sans perçage, 4 prises, une charge jusqu’à 110 kg, une largeur de cadre de 70 à 95 cm et une garantie de 5 ans.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -13913,7 +13991,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c2e6940412c4221"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47c9c67981fb484a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15814,19 +15892,19 @@
       </x:c>
       <x:c r="E25" s="12" t="str">
         <x:f>Produits!E25</x:f>
-        <x:v>KS300</x:v>
+        <x:v>Sportstech KS350</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
         <x:f>Produits!F25</x:f>
         <x:v>Sportstech</x:v>
       </x:c>
-      <x:c r="G25" s="12" t="n">
+      <x:c r="G25" s="12" t="str">
         <x:f>Produits!H25</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H25" s="12" t="n">
+        <x:v>B0843FTZ9T</x:v>
+      </x:c>
+      <x:c r="H25" s="12" t="str">
         <x:f>Produits!I25</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B0843FTZ9T</x:v>
       </x:c>
       <x:c r="I25" s="12" t="n">
         <x:f>Produits!K25</x:f>
@@ -15838,30 +15916,31 @@
       </x:c>
       <x:c r="K25" s="12" t="n">
         <x:f>Produits!U25</x:f>
-        <x:v>0</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="L25" s="12" t="str">
         <x:f>Produits!V25</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="M25" s="12" t="str">
         <x:f>Produits!Z25</x:f>
-        <x:v>Barre polyvalente pour entraînement du haut du corps.</x:v>
+        <x:v>Une barre murale pliable, stable et polyvalente, particulièrement adaptée à un home gym compact.</x:v>
       </x:c>
       <x:c r="N25" s="12" t="str">
         <x:f>Produits!AA25</x:f>
-        <x:v>Multiprises | Polyvalence | Marque connue</x:v>
+        <x:v>Structure acier triangulaire | Pliable jusqu’à 26 cm | 3 positions de prise | 3 œillets d’entraînement | Kit de fixation inclus</x:v>
       </x:c>
       <x:c r="O25" s="12" t="str">
         <x:f>Produits!AB25</x:f>
-        <x:v>Compatibilité porte à vérifier</x:v>
+        <x:v>Perçage obligatoire | Mur solide indispensable | Moins mobile qu’un modèle de porte</x:v>
       </x:c>
       <x:c r="P25" s="12" t="str">
         <x:f>Produits!AC25</x:f>
-        <x:v>Home gym</x:v>
+        <x:v>Débutant à confirmé recherchant une barre murale complète et peu encombrante</x:v>
       </x:c>
       <x:c r="Q25" s="12" t="str">
         <x:f>Produits!AG25</x:f>
-        <x:v>À rechercher</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -15883,19 +15962,19 @@
       </x:c>
       <x:c r="E26" s="12" t="str">
         <x:f>Produits!E26</x:f>
-        <x:v>Wall Mounted Pull-Up Bar</x:v>
+        <x:v>ONETWOFIT OT103</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
         <x:f>Produits!F26</x:f>
         <x:v>ONETWOFIT</x:v>
       </x:c>
-      <x:c r="G26" s="12" t="n">
+      <x:c r="G26" s="12" t="str">
         <x:f>Produits!H26</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H26" s="12" t="n">
+        <x:v>B08K3Q74DR</x:v>
+      </x:c>
+      <x:c r="H26" s="12" t="str">
         <x:f>Produits!I26</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B08K3Q74DR</x:v>
       </x:c>
       <x:c r="I26" s="12" t="n">
         <x:f>Produits!K26</x:f>
@@ -15907,31 +15986,31 @@
       </x:c>
       <x:c r="K26" s="12" t="n">
         <x:f>Produits!U26</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L26" s="12" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="L26" s="12" t="str">
         <x:f>Produits!V26</x:f>
-        <x:v>0</x:v>
+        <x:v>Très bon</x:v>
       </x:c>
       <x:c r="M26" s="12" t="str">
         <x:f>Produits!Z26</x:f>
-        <x:v>Barre murale robuste à prix compétitif.</x:v>
+        <x:v>Une barre murale robuste et accessible, conçue pour offrir une fixation stable sans payer le prix d’un modèle premium.</x:v>
       </x:c>
       <x:c r="N26" s="12" t="str">
         <x:f>Produits!AA26</x:f>
-        <x:v>Stabilité | Multiprises | Prix</x:v>
+        <x:v>Excellent rapport qualité/prix | Conception 6 trous | Multiprises | Utilisation intérieure ou extérieure | Structure acier</x:v>
       </x:c>
       <x:c r="O26" s="12" t="str">
         <x:f>Produits!AB26</x:f>
-        <x:v>Installation avec perçage</x:v>
+        <x:v>Montage mural obligatoire | Qualité des chevilles à adapter au support | Finitions plus simples</x:v>
       </x:c>
       <x:c r="P26" s="12" t="str">
         <x:f>Produits!AC26</x:f>
-        <x:v>Débutant à confirmé</x:v>
+        <x:v>Débutant à intermédiaire souhaitant une solution murale économique</x:v>
       </x:c>
       <x:c r="Q26" s="12" t="str">
         <x:f>Produits!AG26</x:f>
-        <x:v>À rechercher</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -15953,19 +16032,19 @@
       </x:c>
       <x:c r="E27" s="12" t="str">
         <x:f>Produits!E27</x:f>
-        <x:v>Pull-Up &amp; Dip Bar</x:v>
+        <x:v>PULLUP &amp; DIP Barre de traction porte + station de dips</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
         <x:f>Produits!F27</x:f>
-        <x:v>Pullup &amp; Dip</x:v>
-      </x:c>
-      <x:c r="G27" s="12" t="n">
+        <x:v>PULLUP &amp; DIP</x:v>
+      </x:c>
+      <x:c r="G27" s="12" t="str">
         <x:f>Produits!H27</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H27" s="12" t="n">
+        <x:v>B0CGDTN9VC</x:v>
+      </x:c>
+      <x:c r="H27" s="12" t="str">
         <x:f>Produits!I27</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B0CGDTN9VC</x:v>
       </x:c>
       <x:c r="I27" s="12" t="n">
         <x:f>Produits!K27</x:f>
@@ -15975,31 +16054,33 @@
         <x:f>Produits!L27</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K27" s="12" t="str">
+      <x:c r="K27" s="12" t="n">
         <x:f>Produits!U27</x:f>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="L27" s="12" t="str">
         <x:f>Produits!V27</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="M27" s="12" t="str">
         <x:f>Produits!Z27</x:f>
-        <x:v>Solution premium pour calisthénie et usage intensif.</x:v>
+        <x:v>Une solution premium sans perçage qui combine tractions et dips, idéale pour la calisthénie à domicile.</x:v>
       </x:c>
       <x:c r="N27" s="12" t="str">
         <x:f>Produits!AA27</x:f>
-        <x:v>Finition | Polyvalence | Stabilité</x:v>
+        <x:v>Aucun perçage | Barre de dips incluse | 4 positions de prise | Garantie 5 ans | Montage et retrait rapides</x:v>
       </x:c>
       <x:c r="O27" s="12" t="str">
         <x:f>Produits!AB27</x:f>
-        <x:v>Prix élevé</x:v>
+        <x:v>Prix élevé | Compatibilité du cadre de porte à vérifier | Charge limitée à 110 kg</x:v>
       </x:c>
       <x:c r="P27" s="12" t="str">
         <x:f>Produits!AC27</x:f>
-        <x:v>Calisthénie / confirmé</x:v>
+        <x:v>Intermédiaire à confirmé pratiquant la calisthénie ou vivant en location</x:v>
       </x:c>
       <x:c r="Q27" s="12" t="str">
         <x:f>Produits!AG27</x:f>
-        <x:v>À rechercher</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
Import Roues à abdos (validées) + création du comparatif dédié
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQYooFqe2Ca9bkV6gqeZVS
</commit_message>
<xml_diff>
--- a/data/import/MuscuGuide_Base_Produits.xlsx
+++ b/data/import/MuscuGuide_Base_Produits.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R539c652a54024d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="R64f6e295511b429a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="Rdc3186bfebd043f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="Rdc2e9e86ec46411d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="Ra4b4f8a93f0d4617"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="Rb1b39ccfcf3c44d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R92adaef9abe946de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="Rf0202f79178f41e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="R198a761b2c2b434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="R1eb90a37d9054e81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="R7f9ec2f93cd0444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="R44ab3857d0d5419d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -435,7 +435,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R49611829e2f44a32"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc574ed0a565b42b9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -687,7 +687,7 @@
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:f>COUNTA(Produits!E4:E250)</x:f>
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C4" s="12"/>
       <x:c r="D4" s="12" t="str">
@@ -747,7 +747,7 @@
       </x:c>
       <x:c r="B6" s="12" t="n">
         <x:f>COUNTIF(Produits!AG4:AG250,"Validé")</x:f>
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C6" s="12"/>
       <x:c r="D6" s="12" t="str">
@@ -807,7 +807,7 @@
       </x:c>
       <x:c r="B8" s="38" t="n">
         <x:f>IFERROR(AVERAGE(Produits!U4:U250),0)</x:f>
-        <x:v>89.33333333333333</x:v>
+        <x:v>89.53333333333333</x:v>
       </x:c>
       <x:c r="C8" s="12"/>
       <x:c r="D8" s="12" t="str">
@@ -1125,7 +1125,7 @@
       </x:c>
       <x:c r="E19" s="12" t="n">
         <x:f>COUNTIF(Produits!B:B,D19)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F19" s="12" t="n">
         <x:f>COUNTIFS(Produits!B:B,D19,Produits!H:H,"??????????")</x:f>
@@ -1133,7 +1133,7 @@
       </x:c>
       <x:c r="G19" s="12" t="n">
         <x:f>COUNTIFS(Produits!B:B,D19,Produits!AG:AG,"Validé")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H19" s="46" t="n">
         <x:f>IFERROR(F19/E19,0)</x:f>
@@ -1259,7 +1259,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a2e06aea0545b2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b151f4f0c374c5c"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -4849,133 +4849,309 @@
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="12"/>
-      <x:c r="B40" s="12"/>
-      <x:c r="C40" s="12"/>
-      <x:c r="D40" s="12"/>
-      <x:c r="E40" s="12"/>
-      <x:c r="F40" s="12"/>
-      <x:c r="G40" s="12"/>
-      <x:c r="H40" s="12"/>
-      <x:c r="I40" s="12"/>
+      <x:c r="A40" s="12" t="str">
+        <x:v>MG-ROUE-001</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="str">
+        <x:v>Roue à abdos</x:v>
+      </x:c>
+      <x:c r="C40" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D40" s="12" t="str">
+        <x:v>Choix MuscuGuide</x:v>
+      </x:c>
+      <x:c r="E40" s="12" t="str">
+        <x:v>Vinsguir Ab Roller noir/rouge</x:v>
+      </x:c>
+      <x:c r="F40" s="12" t="str">
+        <x:v>Vinsguir</x:v>
+      </x:c>
+      <x:c r="G40" s="12" t="str">
+        <x:v>Roue ultra-large 8 cm — axe acier — tapis pour genoux — charge annoncée 200 kg</x:v>
+      </x:c>
+      <x:c r="H40" s="12" t="str">
+        <x:v>B07RKW5H68</x:v>
+      </x:c>
+      <x:c r="I40" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B07RKW5H68</x:v>
+      </x:c>
       <x:c r="J40" s="12"/>
       <x:c r="K40" s="12" t="str">
         <x:f>IF(OR(H40="",J40=""),"", "https://www.amazon.fr/dp/"&amp;H40&amp;"?tag="&amp;J40)</x:f>
       </x:c>
       <x:c r="L40" s="12"/>
       <x:c r="M40" s="36"/>
-      <x:c r="N40" s="12"/>
-      <x:c r="O40" s="12"/>
-      <x:c r="P40" s="12"/>
-      <x:c r="Q40" s="12"/>
-      <x:c r="R40" s="12"/>
-      <x:c r="S40" s="12"/>
-      <x:c r="T40" s="12"/>
-      <x:c r="U40" s="12" t="str">
+      <x:c r="N40" s="12" t="str">
+        <x:v>Performance</x:v>
+      </x:c>
+      <x:c r="O40" s="12" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P40" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q40" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R40" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="S40" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T40" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="U40" s="12" t="n">
         <x:f>IF(COUNTA(O40:T40)=0,"",SUM(O40:T40))</x:f>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="V40" s="12" t="str">
         <x:f>IF(U40="","",IF(U40&gt;=95,"Exceptionnel",IF(U40&gt;=90,"Excellent",IF(U40&gt;=85,"Très bon",IF(U40&gt;=80,"Bon",IF(U40&gt;=70,"Correct","À revoir"))))))</x:f>
-      </x:c>
-      <x:c r="W40" s="12"/>
-      <x:c r="X40" s="12"/>
-      <x:c r="Y40" s="12"/>
-      <x:c r="Z40" s="12"/>
-      <x:c r="AA40" s="12"/>
-      <x:c r="AB40" s="12"/>
-      <x:c r="AC40" s="12"/>
-      <x:c r="AD40" s="12"/>
-      <x:c r="AE40" s="38"/>
-      <x:c r="AF40" s="40"/>
-      <x:c r="AG40" s="12"/>
-      <x:c r="AH40" s="12"/>
-      <x:c r="AI40" s="12"/>
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="W40" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="X40" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Y40" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Z40" s="12" t="str">
+        <x:v>Une roue abdominale stable, silencieuse et très populaire, adaptée à la majorité des utilisateurs qui souhaitent renforcer leur sangle abdominale à domicile.</x:v>
+      </x:c>
+      <x:c r="AA40" s="12" t="str">
+        <x:v>Roue ultra-large de 8 cm | Plus de 22 000 évaluations | Tapis pour genoux inclus | Fonctionnement silencieux | Charge annoncée jusqu’à 200 kg</x:v>
+      </x:c>
+      <x:c r="AB40" s="12" t="str">
+        <x:v>Poignées en mousse susceptibles de s’user | Pas de résistance assistée | Le mouvement reste exigeant pour un grand débutant</x:v>
+      </x:c>
+      <x:c r="AC40" s="12" t="str">
+        <x:v>Débutant à confirmé recherchant une roue stable et éprouvée</x:v>
+      </x:c>
+      <x:c r="AD40" s="12" t="n">
+        <x:v>22344</x:v>
+      </x:c>
+      <x:c r="AE40" s="38" t="n">
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="AF40" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="AG40" s="12" t="str">
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH40" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B07RKW5H68</x:v>
+      </x:c>
+      <x:c r="AI40" s="12" t="str">
+        <x:v>ASIN, note Amazon 4,6/5 et 22 344 évaluations vérifiés le 05/08/2026. Roue de 8 cm, tapis inclus et charge annoncée 200 kg confirmés par Amazon et Vinsguir : https://myvinsguir.com/</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="12"/>
-      <x:c r="B41" s="12"/>
-      <x:c r="C41" s="12"/>
-      <x:c r="D41" s="12"/>
-      <x:c r="E41" s="12"/>
-      <x:c r="F41" s="12"/>
-      <x:c r="G41" s="12"/>
-      <x:c r="H41" s="12"/>
-      <x:c r="I41" s="12"/>
+      <x:c r="A41" s="12" t="str">
+        <x:v>MG-ROUE-002</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="str">
+        <x:v>Roue à abdos</x:v>
+      </x:c>
+      <x:c r="C41" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D41" s="12" t="str">
+        <x:v>Meilleur rapport qualité/prix</x:v>
+      </x:c>
+      <x:c r="E41" s="12" t="str">
+        <x:v>adidas Ab Wheel 18 cm</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
+        <x:v>adidas</x:v>
+      </x:c>
+      <x:c r="G41" s="12" t="str">
+        <x:v>Diamètre 18 cm — poignées en mousse — surface caoutchoutée antidérapante</x:v>
+      </x:c>
+      <x:c r="H41" s="12" t="str">
+        <x:v>B00EVNXN6K</x:v>
+      </x:c>
+      <x:c r="I41" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B00EVNXN6K</x:v>
+      </x:c>
       <x:c r="J41" s="12"/>
       <x:c r="K41" s="12" t="str">
         <x:f>IF(OR(H41="",J41=""),"", "https://www.amazon.fr/dp/"&amp;H41&amp;"?tag="&amp;J41)</x:f>
       </x:c>
       <x:c r="L41" s="12"/>
       <x:c r="M41" s="36"/>
-      <x:c r="N41" s="12"/>
-      <x:c r="O41" s="12"/>
-      <x:c r="P41" s="12"/>
-      <x:c r="Q41" s="12"/>
-      <x:c r="R41" s="12"/>
-      <x:c r="S41" s="12"/>
-      <x:c r="T41" s="12"/>
-      <x:c r="U41" s="12" t="str">
+      <x:c r="N41" s="12" t="str">
+        <x:v>Essentials</x:v>
+      </x:c>
+      <x:c r="O41" s="12" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P41" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q41" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R41" s="12" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="S41" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T41" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="U41" s="12" t="n">
         <x:f>IF(COUNTA(O41:T41)=0,"",SUM(O41:T41))</x:f>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="V41" s="12" t="str">
         <x:f>IF(U41="","",IF(U41&gt;=95,"Exceptionnel",IF(U41&gt;=90,"Excellent",IF(U41&gt;=85,"Très bon",IF(U41&gt;=80,"Bon",IF(U41&gt;=70,"Correct","À revoir"))))))</x:f>
-      </x:c>
-      <x:c r="W41" s="12"/>
-      <x:c r="X41" s="12"/>
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="W41" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="X41" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
       <x:c r="Y41" s="12"/>
-      <x:c r="Z41" s="12"/>
-      <x:c r="AA41" s="12"/>
-      <x:c r="AB41" s="12"/>
-      <x:c r="AC41" s="12"/>
-      <x:c r="AD41" s="12"/>
-      <x:c r="AE41" s="38"/>
-      <x:c r="AF41" s="40"/>
-      <x:c r="AG41" s="12"/>
-      <x:c r="AH41" s="12"/>
-      <x:c r="AI41" s="12"/>
+      <x:c r="Z41" s="12" t="str">
+        <x:v>Une roue simple, solide et accessible, idéale pour s’équiper avec un produit de marque reconnu sans fonctionnalités superflues.</x:v>
+      </x:c>
+      <x:c r="AA41" s="12" t="str">
+        <x:v>Excellent rapport qualité/prix | Diamètre de 18 cm | Surface caoutchoutée antidérapante | Poignées rembourrées | Près de 9 000 évaluations</x:v>
+      </x:c>
+      <x:c r="AB41" s="12" t="str">
+        <x:v>Montage des poignées parfois difficile | Roue unique moins rassurante au début | Aucun tapis pour genoux inclus</x:v>
+      </x:c>
+      <x:c r="AC41" s="12" t="str">
+        <x:v>Débutant à intermédiaire recherchant une roue simple et durable</x:v>
+      </x:c>
+      <x:c r="AD41" s="12" t="n">
+        <x:v>8992</x:v>
+      </x:c>
+      <x:c r="AE41" s="38" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="AF41" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="AG41" s="12" t="str">
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH41" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B00EVNXN6K</x:v>
+      </x:c>
+      <x:c r="AI41" s="12" t="str">
+        <x:v>ASIN, note Amazon 4,5/5 et 8 992 évaluations vérifiés le 05/08/2026. Diamètre 18 cm, poignées en mousse et surface caoutchoutée confirmés sur Amazon FR.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="12"/>
-      <x:c r="B42" s="12"/>
-      <x:c r="C42" s="12"/>
-      <x:c r="D42" s="12"/>
-      <x:c r="E42" s="12"/>
-      <x:c r="F42" s="12"/>
-      <x:c r="G42" s="12"/>
-      <x:c r="H42" s="12"/>
-      <x:c r="I42" s="12"/>
+      <x:c r="A42" s="12" t="str">
+        <x:v>MG-ROUE-003</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="str">
+        <x:v>Roue à abdos</x:v>
+      </x:c>
+      <x:c r="C42" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D42" s="12" t="str">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="E42" s="12" t="str">
+        <x:v>Perfect Fitness Ab Carver Pro</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
+        <x:v>Perfect Fitness</x:v>
+      </x:c>
+      <x:c r="G42" s="12" t="str">
+        <x:v>Roue ultra-large — ressort interne en acier carbone — poignées ergonomiques — tapis inclus</x:v>
+      </x:c>
+      <x:c r="H42" s="12" t="str">
+        <x:v>B07NCBR97K</x:v>
+      </x:c>
+      <x:c r="I42" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B07NCBR97K</x:v>
+      </x:c>
       <x:c r="J42" s="12"/>
       <x:c r="K42" s="12" t="str">
         <x:f>IF(OR(H42="",J42=""),"", "https://www.amazon.fr/dp/"&amp;H42&amp;"?tag="&amp;J42)</x:f>
       </x:c>
       <x:c r="L42" s="12"/>
       <x:c r="M42" s="36"/>
-      <x:c r="N42" s="12"/>
-      <x:c r="O42" s="12"/>
-      <x:c r="P42" s="12"/>
-      <x:c r="Q42" s="12"/>
-      <x:c r="R42" s="12"/>
-      <x:c r="S42" s="12"/>
-      <x:c r="T42" s="12"/>
-      <x:c r="U42" s="12" t="str">
+      <x:c r="N42" s="12" t="str">
+        <x:v>Elite</x:v>
+      </x:c>
+      <x:c r="O42" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P42" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="Q42" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R42" s="12" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="S42" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T42" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="U42" s="12" t="n">
         <x:f>IF(COUNTA(O42:T42)=0,"",SUM(O42:T42))</x:f>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="V42" s="12" t="str">
         <x:f>IF(U42="","",IF(U42&gt;=95,"Exceptionnel",IF(U42&gt;=90,"Excellent",IF(U42&gt;=85,"Très bon",IF(U42&gt;=80,"Bon",IF(U42&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="W42" s="12"/>
-      <x:c r="X42" s="12"/>
-      <x:c r="Y42" s="12"/>
-      <x:c r="Z42" s="12"/>
-      <x:c r="AA42" s="12"/>
-      <x:c r="AB42" s="12"/>
-      <x:c r="AC42" s="12"/>
-      <x:c r="AD42" s="12"/>
-      <x:c r="AE42" s="38"/>
-      <x:c r="AF42" s="40"/>
-      <x:c r="AG42" s="12"/>
-      <x:c r="AH42" s="12"/>
-      <x:c r="AI42" s="12"/>
+      <x:c r="X42" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Y42" s="12" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="Z42" s="12" t="str">
+        <x:v>Une roue abdominale premium avec résistance intégrée, conçue pour améliorer la stabilité, l’activation musculaire et le contrôle du retour.</x:v>
+      </x:c>
+      <x:c r="AA42" s="12" t="str">
+        <x:v>Résistance à ressort intégrée | Assistance au retour | Roue ultra-large | Travail possible des obliques | Poignées ergonomiques et tapis inclus</x:v>
+      </x:c>
+      <x:c r="AB42" s="12" t="str">
+        <x:v>Prix nettement supérieur | Plus lourde et encombrante | Amplitude potentiellement limitée pour les utilisateurs très grands</x:v>
+      </x:c>
+      <x:c r="AC42" s="12" t="str">
+        <x:v>Intermédiaire à confirmé recherchant davantage de contrôle et de progression</x:v>
+      </x:c>
+      <x:c r="AD42" s="12" t="n">
+        <x:v>13447</x:v>
+      </x:c>
+      <x:c r="AE42" s="38" t="n">
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="AF42" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="AG42" s="12" t="str">
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH42" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B07NCBR97K</x:v>
+      </x:c>
+      <x:c r="AI42" s="12" t="str">
+        <x:v>ASIN, note Amazon 4,6/5 et environ 13 447 évaluations vérifiés le 05/08/2026. Ressort interne, roue ultra-large, poignées ergonomiques et tapis confirmés : https://www.fitnessconcept.com.my/brands/perfect-fitness-ab-carver-pro</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="12"/>
@@ -13991,7 +14167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47c9c67981fb484a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12b0a4b80faf4901"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15845,9 +16021,8 @@
         <x:f>Produits!L24</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K24" s="12" t="n">
+      <x:c r="K24" s="12" t="str">
         <x:f>Produits!U24</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="L24" s="12" t="str">
         <x:f>Produits!V24</x:f>
@@ -16924,37 +17099,37 @@
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="12" t="n">
+      <x:c r="A40" s="12" t="str">
         <x:f>Produits!A40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B40" s="12" t="n">
+        <x:v>MG-ROUE-001</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="str">
         <x:f>Produits!B40</x:f>
-        <x:v>0</x:v>
+        <x:v>Roue à abdos</x:v>
       </x:c>
       <x:c r="C40" s="12" t="n">
         <x:f>Produits!C40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D40" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D40" s="12" t="str">
         <x:f>Produits!D40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E40" s="12" t="n">
+        <x:v>Choix MuscuGuide</x:v>
+      </x:c>
+      <x:c r="E40" s="12" t="str">
         <x:f>Produits!E40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F40" s="12" t="n">
+        <x:v>Vinsguir Ab Roller noir/rouge</x:v>
+      </x:c>
+      <x:c r="F40" s="12" t="str">
         <x:f>Produits!F40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G40" s="12" t="n">
+        <x:v>Vinsguir</x:v>
+      </x:c>
+      <x:c r="G40" s="12" t="str">
         <x:f>Produits!H40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H40" s="12" t="n">
+        <x:v>B07RKW5H68</x:v>
+      </x:c>
+      <x:c r="H40" s="12" t="str">
         <x:f>Produits!I40</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B07RKW5H68</x:v>
       </x:c>
       <x:c r="I40" s="12" t="n">
         <x:f>Produits!K40</x:f>
@@ -16966,65 +17141,65 @@
       </x:c>
       <x:c r="K40" s="12" t="n">
         <x:f>Produits!U40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L40" s="12" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="L40" s="12" t="str">
         <x:f>Produits!V40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M40" s="12" t="n">
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="M40" s="12" t="str">
         <x:f>Produits!Z40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N40" s="12" t="n">
+        <x:v>Une roue abdominale stable, silencieuse et très populaire, adaptée à la majorité des utilisateurs qui souhaitent renforcer leur sangle abdominale à domicile.</x:v>
+      </x:c>
+      <x:c r="N40" s="12" t="str">
         <x:f>Produits!AA40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O40" s="12" t="n">
+        <x:v>Roue ultra-large de 8 cm | Plus de 22 000 évaluations | Tapis pour genoux inclus | Fonctionnement silencieux | Charge annoncée jusqu’à 200 kg</x:v>
+      </x:c>
+      <x:c r="O40" s="12" t="str">
         <x:f>Produits!AB40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P40" s="12" t="n">
+        <x:v>Poignées en mousse susceptibles de s’user | Pas de résistance assistée | Le mouvement reste exigeant pour un grand débutant</x:v>
+      </x:c>
+      <x:c r="P40" s="12" t="str">
         <x:f>Produits!AC40</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q40" s="12" t="n">
+        <x:v>Débutant à confirmé recherchant une roue stable et éprouvée</x:v>
+      </x:c>
+      <x:c r="Q40" s="12" t="str">
         <x:f>Produits!AG40</x:f>
-        <x:v>0</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="12" t="n">
+      <x:c r="A41" s="12" t="str">
         <x:f>Produits!A41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B41" s="12" t="n">
+        <x:v>MG-ROUE-002</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="str">
         <x:f>Produits!B41</x:f>
-        <x:v>0</x:v>
+        <x:v>Roue à abdos</x:v>
       </x:c>
       <x:c r="C41" s="12" t="n">
         <x:f>Produits!C41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D41" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D41" s="12" t="str">
         <x:f>Produits!D41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E41" s="12" t="n">
+        <x:v>Meilleur rapport qualité/prix</x:v>
+      </x:c>
+      <x:c r="E41" s="12" t="str">
         <x:f>Produits!E41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F41" s="12" t="n">
+        <x:v>adidas Ab Wheel 18 cm</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
         <x:f>Produits!F41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G41" s="12" t="n">
+        <x:v>adidas</x:v>
+      </x:c>
+      <x:c r="G41" s="12" t="str">
         <x:f>Produits!H41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H41" s="12" t="n">
+        <x:v>B00EVNXN6K</x:v>
+      </x:c>
+      <x:c r="H41" s="12" t="str">
         <x:f>Produits!I41</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B00EVNXN6K</x:v>
       </x:c>
       <x:c r="I41" s="12" t="n">
         <x:f>Produits!K41</x:f>
@@ -17036,65 +17211,65 @@
       </x:c>
       <x:c r="K41" s="12" t="n">
         <x:f>Produits!U41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L41" s="12" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="L41" s="12" t="str">
         <x:f>Produits!V41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M41" s="12" t="n">
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="M41" s="12" t="str">
         <x:f>Produits!Z41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N41" s="12" t="n">
+        <x:v>Une roue simple, solide et accessible, idéale pour s’équiper avec un produit de marque reconnu sans fonctionnalités superflues.</x:v>
+      </x:c>
+      <x:c r="N41" s="12" t="str">
         <x:f>Produits!AA41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O41" s="12" t="n">
+        <x:v>Excellent rapport qualité/prix | Diamètre de 18 cm | Surface caoutchoutée antidérapante | Poignées rembourrées | Près de 9 000 évaluations</x:v>
+      </x:c>
+      <x:c r="O41" s="12" t="str">
         <x:f>Produits!AB41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P41" s="12" t="n">
+        <x:v>Montage des poignées parfois difficile | Roue unique moins rassurante au début | Aucun tapis pour genoux inclus</x:v>
+      </x:c>
+      <x:c r="P41" s="12" t="str">
         <x:f>Produits!AC41</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q41" s="12" t="n">
+        <x:v>Débutant à intermédiaire recherchant une roue simple et durable</x:v>
+      </x:c>
+      <x:c r="Q41" s="12" t="str">
         <x:f>Produits!AG41</x:f>
-        <x:v>0</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="12" t="n">
+      <x:c r="A42" s="12" t="str">
         <x:f>Produits!A42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B42" s="12" t="n">
+        <x:v>MG-ROUE-003</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="str">
         <x:f>Produits!B42</x:f>
-        <x:v>0</x:v>
+        <x:v>Roue à abdos</x:v>
       </x:c>
       <x:c r="C42" s="12" t="n">
         <x:f>Produits!C42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D42" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D42" s="12" t="str">
         <x:f>Produits!D42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E42" s="12" t="n">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="E42" s="12" t="str">
         <x:f>Produits!E42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F42" s="12" t="n">
+        <x:v>Perfect Fitness Ab Carver Pro</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
         <x:f>Produits!F42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G42" s="12" t="n">
+        <x:v>Perfect Fitness</x:v>
+      </x:c>
+      <x:c r="G42" s="12" t="str">
         <x:f>Produits!H42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H42" s="12" t="n">
+        <x:v>B07NCBR97K</x:v>
+      </x:c>
+      <x:c r="H42" s="12" t="str">
         <x:f>Produits!I42</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B07NCBR97K</x:v>
       </x:c>
       <x:c r="I42" s="12" t="n">
         <x:f>Produits!K42</x:f>
@@ -17106,31 +17281,31 @@
       </x:c>
       <x:c r="K42" s="12" t="n">
         <x:f>Produits!U42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L42" s="12" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="L42" s="12" t="str">
         <x:f>Produits!V42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M42" s="12" t="n">
+        <x:v>Excellent</x:v>
+      </x:c>
+      <x:c r="M42" s="12" t="str">
         <x:f>Produits!Z42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N42" s="12" t="n">
+        <x:v>Une roue abdominale premium avec résistance intégrée, conçue pour améliorer la stabilité, l’activation musculaire et le contrôle du retour.</x:v>
+      </x:c>
+      <x:c r="N42" s="12" t="str">
         <x:f>Produits!AA42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O42" s="12" t="n">
+        <x:v>Résistance à ressort intégrée | Assistance au retour | Roue ultra-large | Travail possible des obliques | Poignées ergonomiques et tapis inclus</x:v>
+      </x:c>
+      <x:c r="O42" s="12" t="str">
         <x:f>Produits!AB42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P42" s="12" t="n">
+        <x:v>Prix nettement supérieur | Plus lourde et encombrante | Amplitude potentiellement limitée pour les utilisateurs très grands</x:v>
+      </x:c>
+      <x:c r="P42" s="12" t="str">
         <x:f>Produits!AC42</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q42" s="12" t="n">
+        <x:v>Intermédiaire à confirmé recherchant davantage de contrôle et de progression</x:v>
+      </x:c>
+      <x:c r="Q42" s="12" t="str">
         <x:f>Produits!AG42</x:f>
-        <x:v>0</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="43">

</xml_diff>

<commit_message>
Import Whey protéine (validées) + branchement du comparatif dédié
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQYooFqe2Ca9bkV6gqeZVS
</commit_message>
<xml_diff>
--- a/data/import/MuscuGuide_Base_Produits.xlsx
+++ b/data/import/MuscuGuide_Base_Produits.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R92adaef9abe946de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="Rf0202f79178f41e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="R198a761b2c2b434f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="R1eb90a37d9054e81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="R7f9ec2f93cd0444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="R44ab3857d0d5419d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R334a96ef688c4e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="2" r:id="Rb4a760d781224aa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notation" sheetId="3" r:id="R90805a10dc074995"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Claude" sheetId="4" r:id="R0191e7c5985e4d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="5" r:id="R481527d990de4ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="6" r:id="R3f19d2b5f82a48ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -435,7 +435,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc574ed0a565b42b9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc556cce810a942f5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -704,7 +704,7 @@
       </x:c>
       <x:c r="G4" s="12" t="n">
         <x:f>COUNTIFS(Produits!B:B,D4,Produits!AG:AG,"Validé")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H4" s="46" t="n">
         <x:f>IFERROR(F4/E4,0)</x:f>
@@ -747,7 +747,7 @@
       </x:c>
       <x:c r="B6" s="12" t="n">
         <x:f>COUNTIF(Produits!AG4:AG250,"Validé")</x:f>
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C6" s="12"/>
       <x:c r="D6" s="12" t="str">
@@ -777,7 +777,7 @@
       </x:c>
       <x:c r="B7" s="12" t="n">
         <x:f>COUNTIF(Produits!AG4:AG250,"À rechercher")</x:f>
-        <x:v>9</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="12"/>
       <x:c r="D7" s="12" t="str">
@@ -807,7 +807,7 @@
       </x:c>
       <x:c r="B8" s="38" t="n">
         <x:f>IFERROR(AVERAGE(Produits!U4:U250),0)</x:f>
-        <x:v>89.53333333333333</x:v>
+        <x:v>89.60606060606061</x:v>
       </x:c>
       <x:c r="C8" s="12"/>
       <x:c r="D8" s="12" t="str">
@@ -1259,7 +1259,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b151f4f0c374c5c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55ef860175db4921"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -1478,14 +1478,20 @@
         <x:v>Choix MuscuGuide</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
-        <x:v>Gold Standard 100% Whey</x:v>
+        <x:v>Optimum Nutrition Gold Standard 100% Whey</x:v>
       </x:c>
       <x:c r="F4" s="12" t="str">
         <x:v>Optimum Nutrition</x:v>
       </x:c>
-      <x:c r="G4" s="12" t="str"/>
-      <x:c r="H4" s="12" t="str"/>
-      <x:c r="I4" s="12" t="str"/>
+      <x:c r="G4" s="12" t="str">
+        <x:v>2,26 kg — Double chocolat riche — 73 doses — 24 g de protéines</x:v>
+      </x:c>
+      <x:c r="H4" s="12" t="str">
+        <x:v>B000QSNYGI</x:v>
+      </x:c>
+      <x:c r="I4" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B000QSNYGI</x:v>
+      </x:c>
       <x:c r="J4" s="12" t="str"/>
       <x:c r="K4" s="12" t="str">
         <x:f>IF(OR(H4="",J4=""),"", "https://www.amazon.fr/dp/"&amp;H4&amp;"?tag="&amp;J4)</x:f>
@@ -1495,17 +1501,31 @@
       <x:c r="N4" s="12" t="str">
         <x:v>Performance</x:v>
       </x:c>
-      <x:c r="O4" s="12" t="str"/>
-      <x:c r="P4" s="12" t="str"/>
-      <x:c r="Q4" s="12" t="str"/>
-      <x:c r="R4" s="12" t="str"/>
-      <x:c r="S4" s="12" t="str"/>
-      <x:c r="T4" s="12" t="str"/>
-      <x:c r="U4" s="12" t="str">
+      <x:c r="O4" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="P4" s="12" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="Q4" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R4" s="12" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="S4" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T4" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="U4" s="12" t="n">
         <x:f>IF(COUNTA(O4:T4)=0,"",SUM(O4:T4))</x:f>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="V4" s="12" t="str">
         <x:f>IF(U4="","",IF(U4&gt;=95,"Exceptionnel",IF(U4&gt;=90,"Excellent",IF(U4&gt;=85,"Très bon",IF(U4&gt;=80,"Bon",IF(U4&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="W4" s="12" t="str">
         <x:v>Oui</x:v>
@@ -1517,26 +1537,34 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="Z4" s="12" t="str">
-        <x:v>Référence polyvalente pour la majorité des pratiquants.</x:v>
+        <x:v>Une whey de référence, facile à intégrer au quotidien et adaptée à la majorité des pratiquants recherchant une formule éprouvée.</x:v>
       </x:c>
       <x:c r="AA4" s="12" t="str">
-        <x:v>Bonne réputation | Formule connue | Large choix</x:v>
+        <x:v>24 g de protéines par portion | 5,5 g de BCAA | Très forte notoriété | Mélange facile | Large choix de saveurs</x:v>
       </x:c>
       <x:c r="AB4" s="12" t="str">
-        <x:v>Prix parfois élevé | Saveurs variables</x:v>
+        <x:v>Prix souvent supérieur aux alternatives | Goût et texture variables selon le parfum | Contient des édulcorants</x:v>
       </x:c>
       <x:c r="AC4" s="12" t="str">
-        <x:v>Débutant à confirmé</x:v>
-      </x:c>
-      <x:c r="AD4" s="12" t="str"/>
-      <x:c r="AE4" s="38" t="str"/>
-      <x:c r="AF4" s="40" t="str"/>
+        <x:v>Débutant à confirmé recherchant une whey polyvalente et reconnue</x:v>
+      </x:c>
+      <x:c r="AD4" s="12" t="n">
+        <x:v>1676</x:v>
+      </x:c>
+      <x:c r="AE4" s="38" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="AF4" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
       <x:c r="AG4" s="12" t="str">
-        <x:v>À rechercher</x:v>
-      </x:c>
-      <x:c r="AH4" s="12" t="str"/>
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH4" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B000QSNYGI</x:v>
+      </x:c>
       <x:c r="AI4" s="12" t="str">
-        <x:v>Sélection éditoriale initiale — vérifier disponibilité Amazon FR.</x:v>
+        <x:v>ASIN, note Amazon 4,5/5 et 1 676 évaluations vérifiés le 05/08/2026. Format 2,26 kg, 73 doses et 24 g de protéines confirmés sur Amazon FR. Formule officielle : https://www.optimumnutrition.com/en-us/products/gold-standard-100-whey-protein-powder</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1553,14 +1581,20 @@
         <x:v>Meilleur rapport qualité/prix</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Critical Whey</x:v>
+        <x:v>Applied Nutrition Critical Whey 2 kg</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>Applied Nutrition</x:v>
       </x:c>
-      <x:c r="G5" s="12" t="str"/>
-      <x:c r="H5" s="12" t="str"/>
-      <x:c r="I5" s="12" t="str"/>
+      <x:c r="G5" s="12" t="str">
+        <x:v>Chocolate Milkshake — 24 g de protéines — 61 portions — 120 kcal</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>B0CN72SD7K</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0CN72SD7K</x:v>
+      </x:c>
       <x:c r="J5" s="12" t="str"/>
       <x:c r="K5" s="12" t="str">
         <x:f>IF(OR(H5="",J5=""),"", "https://www.amazon.fr/dp/"&amp;H5&amp;"?tag="&amp;J5)</x:f>
@@ -1570,17 +1604,31 @@
       <x:c r="N5" s="12" t="str">
         <x:v>Essentials</x:v>
       </x:c>
-      <x:c r="O5" s="12" t="str"/>
-      <x:c r="P5" s="12" t="str"/>
-      <x:c r="Q5" s="12" t="str"/>
-      <x:c r="R5" s="12" t="str"/>
-      <x:c r="S5" s="12" t="str"/>
-      <x:c r="T5" s="12" t="str"/>
-      <x:c r="U5" s="12" t="str">
+      <x:c r="O5" s="12" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="P5" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q5" s="12" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="R5" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="S5" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="T5" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="U5" s="12" t="n">
         <x:f>IF(COUNTA(O5:T5)=0,"",SUM(O5:T5))</x:f>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="V5" s="12" t="str">
         <x:f>IF(U5="","",IF(U5&gt;=95,"Exceptionnel",IF(U5&gt;=90,"Excellent",IF(U5&gt;=85,"Très bon",IF(U5&gt;=80,"Bon",IF(U5&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Très bon</x:v>
       </x:c>
       <x:c r="W5" s="12" t="str">
         <x:v>Oui</x:v>
@@ -1590,26 +1638,34 @@
       </x:c>
       <x:c r="Y5" s="12" t="str"/>
       <x:c r="Z5" s="12" t="str">
-        <x:v>Option accessible pour une consommation régulière.</x:v>
+        <x:v>Une whey accessible et bien dosée, intéressante pour une consommation régulière avec un budget maîtrisé.</x:v>
       </x:c>
       <x:c r="AA5" s="12" t="str">
-        <x:v>Tarif compétitif | Marque connue | Polyvalente</x:v>
+        <x:v>24 g de protéines | Bon rapport quantité/prix | 61 portions | 120 kcal par portion | BCAA et glutamine</x:v>
       </x:c>
       <x:c r="AB5" s="12" t="str">
-        <x:v>Composition à comparer selon parfum</x:v>
+        <x:v>Note client plus basse que les références premium | Composition pouvant varier selon le parfum | Texture plus sucrée pour certains utilisateurs</x:v>
       </x:c>
       <x:c r="AC5" s="12" t="str">
-        <x:v>Débutant / intermédiaire</x:v>
-      </x:c>
-      <x:c r="AD5" s="12" t="str"/>
-      <x:c r="AE5" s="38" t="str"/>
-      <x:c r="AF5" s="40" t="str"/>
+        <x:v>Débutant à intermédiaire recherchant une whey économique pour un usage régulier</x:v>
+      </x:c>
+      <x:c r="AD5" s="12" t="n">
+        <x:v>1465</x:v>
+      </x:c>
+      <x:c r="AE5" s="38" t="n">
+        <x:v>4.2</x:v>
+      </x:c>
+      <x:c r="AF5" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
       <x:c r="AG5" s="12" t="str">
-        <x:v>À rechercher</x:v>
-      </x:c>
-      <x:c r="AH5" s="12" t="str"/>
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH5" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B0CN72SD7K</x:v>
+      </x:c>
       <x:c r="AI5" s="12" t="str">
-        <x:v>Sélection éditoriale initiale.</x:v>
+        <x:v>ASIN, note Amazon 4,2/5 et 1 465 évaluations vérifiés le 05/08/2026. La formule actuelle annonce 24 g de protéines, 61 portions et 120 kcal : https://appliednutrition.uk/products/critical-whey</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1626,14 +1682,20 @@
         <x:v>Premium</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>Iso Whey Zero</x:v>
+        <x:v>BioTechUSA Iso Whey Zero 908 g</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
         <x:v>BioTechUSA</x:v>
       </x:c>
-      <x:c r="G6" s="12" t="str"/>
-      <x:c r="H6" s="12" t="str"/>
-      <x:c r="I6" s="12" t="str"/>
+      <x:c r="G6" s="12" t="str">
+        <x:v>Black Biscuit — isolat — 21 g de protéines — lactose réduit — sans sucres</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="str">
+        <x:v>B08TWSPB1F</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B08TWSPB1F</x:v>
+      </x:c>
       <x:c r="J6" s="12" t="str"/>
       <x:c r="K6" s="12" t="str">
         <x:f>IF(OR(H6="",J6=""),"", "https://www.amazon.fr/dp/"&amp;H6&amp;"?tag="&amp;J6)</x:f>
@@ -1643,17 +1705,31 @@
       <x:c r="N6" s="12" t="str">
         <x:v>Elite</x:v>
       </x:c>
-      <x:c r="O6" s="12" t="str"/>
-      <x:c r="P6" s="12" t="str"/>
-      <x:c r="Q6" s="12" t="str"/>
-      <x:c r="R6" s="12" t="str"/>
-      <x:c r="S6" s="12" t="str"/>
-      <x:c r="T6" s="12" t="str"/>
-      <x:c r="U6" s="12" t="str">
+      <x:c r="O6" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P6" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="Q6" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="R6" s="12" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="S6" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="T6" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="U6" s="12" t="n">
         <x:f>IF(COUNTA(O6:T6)=0,"",SUM(O6:T6))</x:f>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="V6" s="12" t="str">
         <x:f>IF(U6="","",IF(U6&gt;=95,"Exceptionnel",IF(U6&gt;=90,"Excellent",IF(U6&gt;=85,"Très bon",IF(U6&gt;=80,"Bon",IF(U6&gt;=70,"Correct","À revoir"))))))</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="W6" s="12" t="str"/>
       <x:c r="X6" s="12" t="str">
@@ -1663,26 +1739,34 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="Z6" s="12" t="str">
-        <x:v>Isolat premium pour les utilisateurs exigeants.</x:v>
+        <x:v>Un isolat premium destiné aux utilisateurs qui privilégient une formule riche en protéines, pauvre en sucres et à teneur réduite en lactose.</x:v>
       </x:c>
       <x:c r="AA6" s="12" t="str">
-        <x:v>Faible teneur en sucres | Formule isolat | Image premium</x:v>
+        <x:v>Isolat de whey | 21 g de protéines par portion | Teneur réduite en lactose | Sans sucres et sans gluten | BCAA et glutamine ajoutés</x:v>
       </x:c>
       <x:c r="AB6" s="12" t="str">
-        <x:v>Prix élevé</x:v>
+        <x:v>Prix élevé au kilogramme | Format de 908 g plus petit | Saveurs parfois très marquées</x:v>
       </x:c>
       <x:c r="AC6" s="12" t="str">
-        <x:v>Intermédiaire / confirmé</x:v>
-      </x:c>
-      <x:c r="AD6" s="12" t="str"/>
-      <x:c r="AE6" s="38" t="str"/>
-      <x:c r="AF6" s="40" t="str"/>
+        <x:v>Intermédiaire à confirmé recherchant un isolat premium et une formule allégée en sucres</x:v>
+      </x:c>
+      <x:c r="AD6" s="12" t="n">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="AE6" s="38" t="n">
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="AF6" s="55" t="n">
+        <x:v>46239</x:v>
+      </x:c>
       <x:c r="AG6" s="12" t="str">
-        <x:v>À rechercher</x:v>
-      </x:c>
-      <x:c r="AH6" s="12" t="str"/>
+        <x:v>Validé</x:v>
+      </x:c>
+      <x:c r="AH6" s="12" t="str">
+        <x:v>https://www.amazon.fr/dp/B08TWSPB1F</x:v>
+      </x:c>
       <x:c r="AI6" s="12" t="str">
-        <x:v>Sélection éditoriale initiale.</x:v>
+        <x:v>ASIN, note Amazon 4,6/5 et 171 évaluations vérifiés le 05/08/2026. Amazon FR annonce 21 g de protéines par portion, une teneur réduite en lactose, sans sucres et sans gluten. Source officielle : https://shop.biotechusa.com/products/iso-whey-zero-1816-g</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -14167,7 +14251,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12b0a4b80faf4901"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc30f7ec191d4b86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14605,19 +14689,19 @@
       </x:c>
       <x:c r="E4" s="12" t="str">
         <x:f>Produits!E4</x:f>
-        <x:v>Gold Standard 100% Whey</x:v>
+        <x:v>Optimum Nutrition Gold Standard 100% Whey</x:v>
       </x:c>
       <x:c r="F4" s="12" t="str">
         <x:f>Produits!F4</x:f>
         <x:v>Optimum Nutrition</x:v>
       </x:c>
-      <x:c r="G4" s="12" t="n">
+      <x:c r="G4" s="12" t="str">
         <x:f>Produits!H4</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H4" s="12" t="n">
+        <x:v>B000QSNYGI</x:v>
+      </x:c>
+      <x:c r="H4" s="12" t="str">
         <x:f>Produits!I4</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B000QSNYGI</x:v>
       </x:c>
       <x:c r="I4" s="12" t="n">
         <x:f>Produits!K4</x:f>
@@ -14629,30 +14713,31 @@
       </x:c>
       <x:c r="K4" s="12" t="n">
         <x:f>Produits!U4</x:f>
-        <x:v>0</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="L4" s="12" t="str">
         <x:f>Produits!V4</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="M4" s="12" t="str">
         <x:f>Produits!Z4</x:f>
-        <x:v>Référence polyvalente pour la majorité des pratiquants.</x:v>
+        <x:v>Une whey de référence, facile à intégrer au quotidien et adaptée à la majorité des pratiquants recherchant une formule éprouvée.</x:v>
       </x:c>
       <x:c r="N4" s="12" t="str">
         <x:f>Produits!AA4</x:f>
-        <x:v>Bonne réputation | Formule connue | Large choix</x:v>
+        <x:v>24 g de protéines par portion | 5,5 g de BCAA | Très forte notoriété | Mélange facile | Large choix de saveurs</x:v>
       </x:c>
       <x:c r="O4" s="12" t="str">
         <x:f>Produits!AB4</x:f>
-        <x:v>Prix parfois élevé | Saveurs variables</x:v>
+        <x:v>Prix souvent supérieur aux alternatives | Goût et texture variables selon le parfum | Contient des édulcorants</x:v>
       </x:c>
       <x:c r="P4" s="12" t="str">
         <x:f>Produits!AC4</x:f>
-        <x:v>Débutant à confirmé</x:v>
+        <x:v>Débutant à confirmé recherchant une whey polyvalente et reconnue</x:v>
       </x:c>
       <x:c r="Q4" s="12" t="str">
         <x:f>Produits!AG4</x:f>
-        <x:v>À rechercher</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -14674,19 +14759,19 @@
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:f>Produits!E5</x:f>
-        <x:v>Critical Whey</x:v>
+        <x:v>Applied Nutrition Critical Whey 2 kg</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:f>Produits!F5</x:f>
         <x:v>Applied Nutrition</x:v>
       </x:c>
-      <x:c r="G5" s="12" t="n">
+      <x:c r="G5" s="12" t="str">
         <x:f>Produits!H5</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H5" s="12" t="n">
+        <x:v>B0CN72SD7K</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
         <x:f>Produits!I5</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B0CN72SD7K</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>Produits!K5</x:f>
@@ -14698,31 +14783,31 @@
       </x:c>
       <x:c r="K5" s="12" t="n">
         <x:f>Produits!U5</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L5" s="12" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="L5" s="12" t="str">
         <x:f>Produits!V5</x:f>
-        <x:v>0</x:v>
+        <x:v>Très bon</x:v>
       </x:c>
       <x:c r="M5" s="12" t="str">
         <x:f>Produits!Z5</x:f>
-        <x:v>Option accessible pour une consommation régulière.</x:v>
+        <x:v>Une whey accessible et bien dosée, intéressante pour une consommation régulière avec un budget maîtrisé.</x:v>
       </x:c>
       <x:c r="N5" s="12" t="str">
         <x:f>Produits!AA5</x:f>
-        <x:v>Tarif compétitif | Marque connue | Polyvalente</x:v>
+        <x:v>24 g de protéines | Bon rapport quantité/prix | 61 portions | 120 kcal par portion | BCAA et glutamine</x:v>
       </x:c>
       <x:c r="O5" s="12" t="str">
         <x:f>Produits!AB5</x:f>
-        <x:v>Composition à comparer selon parfum</x:v>
+        <x:v>Note client plus basse que les références premium | Composition pouvant varier selon le parfum | Texture plus sucrée pour certains utilisateurs</x:v>
       </x:c>
       <x:c r="P5" s="12" t="str">
         <x:f>Produits!AC5</x:f>
-        <x:v>Débutant / intermédiaire</x:v>
+        <x:v>Débutant à intermédiaire recherchant une whey économique pour un usage régulier</x:v>
       </x:c>
       <x:c r="Q5" s="12" t="str">
         <x:f>Produits!AG5</x:f>
-        <x:v>À rechercher</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -14744,19 +14829,19 @@
       </x:c>
       <x:c r="E6" s="12" t="str">
         <x:f>Produits!E6</x:f>
-        <x:v>Iso Whey Zero</x:v>
+        <x:v>BioTechUSA Iso Whey Zero 908 g</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
         <x:f>Produits!F6</x:f>
         <x:v>BioTechUSA</x:v>
       </x:c>
-      <x:c r="G6" s="12" t="n">
+      <x:c r="G6" s="12" t="str">
         <x:f>Produits!H6</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H6" s="12" t="n">
+        <x:v>B08TWSPB1F</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="str">
         <x:f>Produits!I6</x:f>
-        <x:v>0</x:v>
+        <x:v>https://www.amazon.fr/dp/B08TWSPB1F</x:v>
       </x:c>
       <x:c r="I6" s="12" t="n">
         <x:f>Produits!K6</x:f>
@@ -14768,30 +14853,31 @@
       </x:c>
       <x:c r="K6" s="12" t="n">
         <x:f>Produits!U6</x:f>
-        <x:v>0</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="L6" s="12" t="str">
         <x:f>Produits!V6</x:f>
+        <x:v>Excellent</x:v>
       </x:c>
       <x:c r="M6" s="12" t="str">
         <x:f>Produits!Z6</x:f>
-        <x:v>Isolat premium pour les utilisateurs exigeants.</x:v>
+        <x:v>Un isolat premium destiné aux utilisateurs qui privilégient une formule riche en protéines, pauvre en sucres et à teneur réduite en lactose.</x:v>
       </x:c>
       <x:c r="N6" s="12" t="str">
         <x:f>Produits!AA6</x:f>
-        <x:v>Faible teneur en sucres | Formule isolat | Image premium</x:v>
+        <x:v>Isolat de whey | 21 g de protéines par portion | Teneur réduite en lactose | Sans sucres et sans gluten | BCAA et glutamine ajoutés</x:v>
       </x:c>
       <x:c r="O6" s="12" t="str">
         <x:f>Produits!AB6</x:f>
-        <x:v>Prix élevé</x:v>
+        <x:v>Prix élevé au kilogramme | Format de 908 g plus petit | Saveurs parfois très marquées</x:v>
       </x:c>
       <x:c r="P6" s="12" t="str">
         <x:f>Produits!AC6</x:f>
-        <x:v>Intermédiaire / confirmé</x:v>
+        <x:v>Intermédiaire à confirmé recherchant un isolat premium et une formule allégée en sucres</x:v>
       </x:c>
       <x:c r="Q6" s="12" t="str">
         <x:f>Produits!AG6</x:f>
-        <x:v>À rechercher</x:v>
+        <x:v>Validé</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>